<commit_message>
US-15129 [IMP] MSR: Adding XLSX reports instead of XLS/CSV
Signed-off-by: Dorian Kemps <dk@tempo-consulting.fr>
</commit_message>
<xml_diff>
--- a/bin/addons/mission_stock/report/consolidated_mission_stock_report.xlsx
+++ b/bin/addons/mission_stock/report/consolidated_mission_stock_report.xlsx
@@ -262,7 +262,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="dd/mmm/yyyy\ hh:mm"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.00###"/>
+    <numFmt numFmtId="166" formatCode="0.00###"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -275,7 +275,7 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -353,6 +353,9 @@
     <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -360,9 +363,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -739,125 +739,125 @@
       </c>
     </row>
     <row r="4" spans="1:119" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="I4" s="8" t="s">
+      <c r="I4" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="J4" s="8"/>
-      <c r="K4" s="8"/>
-      <c r="L4" s="8"/>
-      <c r="M4" s="8"/>
-      <c r="N4" s="8"/>
-      <c r="O4" s="8"/>
-      <c r="P4" s="8"/>
-      <c r="Q4" s="8"/>
-      <c r="R4" s="8"/>
-      <c r="S4" s="8"/>
-      <c r="T4" s="8"/>
-      <c r="U4" s="8"/>
-      <c r="V4" s="8"/>
-      <c r="W4" s="8"/>
-      <c r="X4" s="8"/>
-      <c r="Y4" s="8"/>
-      <c r="Z4" s="8"/>
-      <c r="AA4" s="8"/>
-      <c r="AB4" s="8"/>
-      <c r="AC4" s="8"/>
-      <c r="AD4" s="8"/>
-      <c r="AE4" s="8"/>
-      <c r="AF4" s="8"/>
-      <c r="AG4" s="8"/>
-      <c r="AH4" s="8"/>
-      <c r="AI4" s="8"/>
-      <c r="AJ4" s="8"/>
-      <c r="AK4" s="8"/>
-      <c r="AL4" s="8"/>
-      <c r="AM4" s="8"/>
-      <c r="AN4" s="9" t="s">
+      <c r="J4" s="9"/>
+      <c r="K4" s="9"/>
+      <c r="L4" s="9"/>
+      <c r="M4" s="9"/>
+      <c r="N4" s="9"/>
+      <c r="O4" s="9"/>
+      <c r="P4" s="9"/>
+      <c r="Q4" s="9"/>
+      <c r="R4" s="9"/>
+      <c r="S4" s="9"/>
+      <c r="T4" s="9"/>
+      <c r="U4" s="9"/>
+      <c r="V4" s="9"/>
+      <c r="W4" s="9"/>
+      <c r="X4" s="9"/>
+      <c r="Y4" s="9"/>
+      <c r="Z4" s="9"/>
+      <c r="AA4" s="9"/>
+      <c r="AB4" s="9"/>
+      <c r="AC4" s="9"/>
+      <c r="AD4" s="9"/>
+      <c r="AE4" s="9"/>
+      <c r="AF4" s="9"/>
+      <c r="AG4" s="9"/>
+      <c r="AH4" s="9"/>
+      <c r="AI4" s="9"/>
+      <c r="AJ4" s="9"/>
+      <c r="AK4" s="9"/>
+      <c r="AL4" s="9"/>
+      <c r="AM4" s="9"/>
+      <c r="AN4" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="AO4" s="9"/>
-      <c r="AP4" s="9"/>
-      <c r="AQ4" s="9"/>
-      <c r="AR4" s="9"/>
-      <c r="AS4" s="9"/>
-      <c r="AT4" s="9"/>
-      <c r="AU4" s="9"/>
-      <c r="AV4" s="9"/>
-      <c r="AW4" s="9"/>
-      <c r="AX4" s="9"/>
-      <c r="AY4" s="9"/>
-      <c r="AZ4" s="9"/>
-      <c r="BA4" s="9"/>
-      <c r="BB4" s="9"/>
-      <c r="BC4" s="9"/>
-      <c r="BD4" s="9"/>
-      <c r="BE4" s="9"/>
-      <c r="BF4" s="9"/>
-      <c r="BG4" s="9"/>
-      <c r="BH4" s="9"/>
-      <c r="BI4" s="9"/>
-      <c r="BJ4" s="9"/>
-      <c r="BK4" s="9"/>
-      <c r="BL4" s="9"/>
-      <c r="BM4" s="9"/>
-      <c r="BN4" s="9"/>
-      <c r="BO4" s="9"/>
-      <c r="BP4" s="8" t="s">
+      <c r="AO4" s="10"/>
+      <c r="AP4" s="10"/>
+      <c r="AQ4" s="10"/>
+      <c r="AR4" s="10"/>
+      <c r="AS4" s="10"/>
+      <c r="AT4" s="10"/>
+      <c r="AU4" s="10"/>
+      <c r="AV4" s="10"/>
+      <c r="AW4" s="10"/>
+      <c r="AX4" s="10"/>
+      <c r="AY4" s="10"/>
+      <c r="AZ4" s="10"/>
+      <c r="BA4" s="10"/>
+      <c r="BB4" s="10"/>
+      <c r="BC4" s="10"/>
+      <c r="BD4" s="10"/>
+      <c r="BE4" s="10"/>
+      <c r="BF4" s="10"/>
+      <c r="BG4" s="10"/>
+      <c r="BH4" s="10"/>
+      <c r="BI4" s="10"/>
+      <c r="BJ4" s="10"/>
+      <c r="BK4" s="10"/>
+      <c r="BL4" s="10"/>
+      <c r="BM4" s="10"/>
+      <c r="BN4" s="10"/>
+      <c r="BO4" s="10"/>
+      <c r="BP4" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="BQ4" s="8"/>
-      <c r="BR4" s="8"/>
-      <c r="BS4" s="8"/>
-      <c r="BT4" s="8"/>
-      <c r="BU4" s="8"/>
-      <c r="BV4" s="8"/>
-      <c r="BW4" s="8"/>
-      <c r="BX4" s="8"/>
-      <c r="BY4" s="8"/>
-      <c r="BZ4" s="8"/>
-      <c r="CA4" s="8"/>
-      <c r="CB4" s="8"/>
-      <c r="CC4" s="8"/>
-      <c r="CD4" s="8"/>
-      <c r="CE4" s="8"/>
-      <c r="CF4" s="8"/>
-      <c r="CG4" s="8"/>
-      <c r="CH4" s="8"/>
-      <c r="CI4" s="8"/>
-      <c r="CJ4" s="8"/>
-      <c r="CK4" s="8"/>
-      <c r="CL4" s="8"/>
-      <c r="CM4" s="8"/>
-      <c r="CN4" s="8"/>
-      <c r="CO4" s="10" t="s">
+      <c r="BQ4" s="9"/>
+      <c r="BR4" s="9"/>
+      <c r="BS4" s="9"/>
+      <c r="BT4" s="9"/>
+      <c r="BU4" s="9"/>
+      <c r="BV4" s="9"/>
+      <c r="BW4" s="9"/>
+      <c r="BX4" s="9"/>
+      <c r="BY4" s="9"/>
+      <c r="BZ4" s="9"/>
+      <c r="CA4" s="9"/>
+      <c r="CB4" s="9"/>
+      <c r="CC4" s="9"/>
+      <c r="CD4" s="9"/>
+      <c r="CE4" s="9"/>
+      <c r="CF4" s="9"/>
+      <c r="CG4" s="9"/>
+      <c r="CH4" s="9"/>
+      <c r="CI4" s="9"/>
+      <c r="CJ4" s="9"/>
+      <c r="CK4" s="9"/>
+      <c r="CL4" s="9"/>
+      <c r="CM4" s="9"/>
+      <c r="CN4" s="9"/>
+      <c r="CO4" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="CP4" s="10"/>
-      <c r="CQ4" s="10"/>
-      <c r="CR4" s="10"/>
-      <c r="CS4" s="10"/>
-      <c r="CT4" s="10"/>
-      <c r="CU4" s="10"/>
-      <c r="CV4" s="10"/>
-      <c r="CW4" s="10"/>
-      <c r="CX4" s="10"/>
-      <c r="CY4" s="10"/>
-      <c r="CZ4" s="10"/>
-      <c r="DA4" s="10"/>
-      <c r="DB4" s="10"/>
-      <c r="DC4" s="10"/>
-      <c r="DD4" s="10"/>
-      <c r="DE4" s="10"/>
-      <c r="DF4" s="10"/>
-      <c r="DG4" s="10"/>
-      <c r="DH4" s="10"/>
-      <c r="DI4" s="10"/>
-      <c r="DJ4" s="10"/>
-      <c r="DK4" s="10"/>
-      <c r="DL4" s="10"/>
-      <c r="DM4" s="10"/>
-      <c r="DN4" s="10"/>
-      <c r="DO4" s="10"/>
+      <c r="CP4" s="11"/>
+      <c r="CQ4" s="11"/>
+      <c r="CR4" s="11"/>
+      <c r="CS4" s="11"/>
+      <c r="CT4" s="11"/>
+      <c r="CU4" s="11"/>
+      <c r="CV4" s="11"/>
+      <c r="CW4" s="11"/>
+      <c r="CX4" s="11"/>
+      <c r="CY4" s="11"/>
+      <c r="CZ4" s="11"/>
+      <c r="DA4" s="11"/>
+      <c r="DB4" s="11"/>
+      <c r="DC4" s="11"/>
+      <c r="DD4" s="11"/>
+      <c r="DE4" s="11"/>
+      <c r="DF4" s="11"/>
+      <c r="DG4" s="11"/>
+      <c r="DH4" s="11"/>
+      <c r="DI4" s="11"/>
+      <c r="DJ4" s="11"/>
+      <c r="DK4" s="11"/>
+      <c r="DL4" s="11"/>
+      <c r="DM4" s="11"/>
+      <c r="DN4" s="11"/>
+      <c r="DO4" s="11"/>
     </row>
     <row r="5" spans="1:119" ht="45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
@@ -1233,14 +1233,14 @@
       <c r="F6" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="8">
         <v>5.4927799999999998</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>63</v>
       </c>
       <c r="I6" s="7"/>
-      <c r="J6" s="11"/>
+      <c r="J6" s="8"/>
       <c r="K6" s="7"/>
       <c r="L6" s="7"/>
       <c r="M6" s="7"/>
@@ -1368,14 +1368,14 @@
       <c r="F7" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="8">
         <v>1</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>63</v>
       </c>
       <c r="I7" s="7"/>
-      <c r="J7" s="11"/>
+      <c r="J7" s="8"/>
       <c r="K7" s="7"/>
       <c r="L7" s="7"/>
       <c r="M7" s="7"/>
@@ -1501,14 +1501,14 @@
       <c r="F8" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G8" s="11">
+      <c r="G8" s="8">
         <v>1</v>
       </c>
       <c r="H8" s="1" t="s">
         <v>63</v>
       </c>
       <c r="I8" s="7"/>
-      <c r="J8" s="11"/>
+      <c r="J8" s="8"/>
       <c r="K8" s="7"/>
       <c r="L8" s="7"/>
       <c r="M8" s="7"/>
@@ -1634,7 +1634,7 @@
       <c r="F9" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G9" s="11">
+      <c r="G9" s="8">
         <v>19.97</v>
       </c>
       <c r="H9" s="1" t="s">
@@ -1643,7 +1643,7 @@
       <c r="I9" s="7">
         <v>7</v>
       </c>
-      <c r="J9" s="11">
+      <c r="J9" s="8">
         <v>139.79</v>
       </c>
       <c r="K9" s="7"/>
@@ -1779,14 +1779,14 @@
       <c r="F10" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G10" s="11">
+      <c r="G10" s="8">
         <v>4.79</v>
       </c>
       <c r="H10" s="1" t="s">
         <v>63</v>
       </c>
       <c r="I10" s="7"/>
-      <c r="J10" s="11"/>
+      <c r="J10" s="8"/>
       <c r="K10" s="7"/>
       <c r="L10" s="7"/>
       <c r="M10" s="7"/>
@@ -1914,14 +1914,14 @@
       <c r="F11" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G11" s="11">
+      <c r="G11" s="8">
         <v>0.41</v>
       </c>
       <c r="H11" s="1" t="s">
         <v>63</v>
       </c>
       <c r="I11" s="7"/>
-      <c r="J11" s="11"/>
+      <c r="J11" s="8"/>
       <c r="K11" s="7"/>
       <c r="L11" s="7"/>
       <c r="M11" s="7"/>
@@ -2049,14 +2049,14 @@
       <c r="F12" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="G12" s="11">
+      <c r="G12" s="8">
         <v>1</v>
       </c>
       <c r="H12" s="1" t="s">
         <v>63</v>
       </c>
       <c r="I12" s="7"/>
-      <c r="J12" s="11"/>
+      <c r="J12" s="8"/>
       <c r="K12" s="7"/>
       <c r="L12" s="7"/>
       <c r="M12" s="7"/>

</xml_diff>